<commit_message>
Wave 1 complete: add findings #13–25 to Excel tracker
New Wave 1 failures and fishies (Batches 6–21):
  #13 trigger_flow/test_flow — sys_hub_flow_trigger invalid
  #14 list/get/create_subflow — sys_hub_subflow invalid
  #15 list_portal_pages — sp_portal filter ignored
  #16 list_ux_pages — ux_app_config filter ignored
  #17 get_event_registry_entry — name vs event_name field
  #18 register_event — name vs event_name field
  #19 list_homepages — sys_ui_hp invalid
  #20 list_pa_jobs/get_pa_job — pa_job invalid
  #21 export_properties — category filter ignored
  #22 get_va_conversation — sys_cs_conversation_message invalid
  #23 list_va_categories — sys_cs_category invalid
  #24 get_performance_analytics — pa_job_log fallback invalid
  #25 ml_model_training_history — ml_solution_version invalid

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/solvvision/solvvision-mcp-findings.xlsx
+++ b/solvvision/solvvision-mcp-findings.xlsx
@@ -991,7 +991,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M274"/>
+  <dimension ref="A1:M287"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -18290,6 +18290,851 @@
       <c r="M274" s="3" t="inlineStr">
         <is>
           <t>Spurious guard removed in wave-1-low-complexity-fixes branch</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="n">
+        <v>13</v>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>trigger_flow / test_flow — Invalid table sys_hub_flow_trigger does not exist</t>
+        </is>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>flow</t>
+        </is>
+      </c>
+      <c r="D275" t="inlineStr">
+        <is>
+          <t>trigger_flow, test_flow</t>
+        </is>
+      </c>
+      <c r="E275" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="F275" t="inlineStr">
+        <is>
+          <t>Wrong table name</t>
+        </is>
+      </c>
+      <c r="G275" t="inlineStr">
+        <is>
+          <t>Wave 1</t>
+        </is>
+      </c>
+      <c r="H275" t="inlineStr">
+        <is>
+          <t>Flows must be triggered via REST API endpoint (POST /api/now/flow_api/...) not via Table API insert into sys_hub_flow_trigger. Rewrite handler to use the Flow Designer REST API.</t>
+        </is>
+      </c>
+      <c r="I275" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J275" t="inlineStr">
+        <is>
+          <t>Fork</t>
+        </is>
+      </c>
+      <c r="K275" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="L275" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="M275" t="inlineStr">
+        <is>
+          <t>sys_hub_flow_trigger is not a writable ServiceNow table. Flow triggering requires the Flow Designer API.</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="n">
+        <v>14</v>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>list_subflows / get_subflow / create_subflow — Invalid table sys_hub_subflow does not exist</t>
+        </is>
+      </c>
+      <c r="C276" t="inlineStr">
+        <is>
+          <t>flow</t>
+        </is>
+      </c>
+      <c r="D276" t="inlineStr">
+        <is>
+          <t>list_subflows, get_subflow, create_subflow</t>
+        </is>
+      </c>
+      <c r="E276" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="F276" t="inlineStr">
+        <is>
+          <t>Wrong table name</t>
+        </is>
+      </c>
+      <c r="G276" t="inlineStr">
+        <is>
+          <t>Wave 1</t>
+        </is>
+      </c>
+      <c r="H276" t="inlineStr">
+        <is>
+          <t>Subflows are stored in sys_hub_flow with type=subflow. Change all three handlers to query sys_hub_flow with ^type=subflow appended to the encoded query.</t>
+        </is>
+      </c>
+      <c r="I276" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J276" t="inlineStr">
+        <is>
+          <t>Fork</t>
+        </is>
+      </c>
+      <c r="K276" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="L276" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="M276" t="inlineStr">
+        <is>
+          <t>sys_hub_subflow is not a ServiceNow table. Both list and get must filter sys_hub_flow by type=subflow.</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="n">
+        <v>15</v>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>list_portal_pages — sp_portal filter silently ignored; returns all pages</t>
+        </is>
+      </c>
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="D277" t="inlineStr">
+        <is>
+          <t>list_portal_pages</t>
+        </is>
+      </c>
+      <c r="E277" t="inlineStr">
+        <is>
+          <t>Fishy</t>
+        </is>
+      </c>
+      <c r="F277" t="inlineStr">
+        <is>
+          <t>Wrong filter field</t>
+        </is>
+      </c>
+      <c r="G277" t="inlineStr">
+        <is>
+          <t>Wave 1</t>
+        </is>
+      </c>
+      <c r="H277" t="inlineStr">
+        <is>
+          <t>Verify that the encoded query uses sp_portal=&lt;sys_id&gt; (the reference field on sp_page). If the handler uses portal= or portal_id=, correct to sp_portal=.</t>
+        </is>
+      </c>
+      <c r="I277" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J277" t="inlineStr">
+        <is>
+          <t>Fork</t>
+        </is>
+      </c>
+      <c r="K277" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="L277" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="M277" t="inlineStr">
+        <is>
+          <t>50 records returned when filtering by newly-created portal; expected 0. Filter field name mismatch suspected.</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="n">
+        <v>16</v>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>list_ux_pages — ux_app_config filter silently ignored; returns all pages</t>
+        </is>
+      </c>
+      <c r="C278" t="inlineStr">
+        <is>
+          <t>portal</t>
+        </is>
+      </c>
+      <c r="D278" t="inlineStr">
+        <is>
+          <t>list_ux_pages</t>
+        </is>
+      </c>
+      <c r="E278" t="inlineStr">
+        <is>
+          <t>Fishy</t>
+        </is>
+      </c>
+      <c r="F278" t="inlineStr">
+        <is>
+          <t>Wrong filter field</t>
+        </is>
+      </c>
+      <c r="G278" t="inlineStr">
+        <is>
+          <t>Wave 1</t>
+        </is>
+      </c>
+      <c r="H278" t="inlineStr">
+        <is>
+          <t>Verify the encoded query field for UX app filtering on sys_ux_page. The field may be sys_scope or application, not ux_app_config.</t>
+        </is>
+      </c>
+      <c r="I278" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J278" t="inlineStr">
+        <is>
+          <t>Fork</t>
+        </is>
+      </c>
+      <c r="K278" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="L278" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="M278" t="inlineStr">
+        <is>
+          <t>22 records returned when filtering by fake app_sys_id; expected 0. Filter field likely wrong.</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="n">
+        <v>17</v>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>get_event_registry_entry — filter uses wrong field name; returns first record regardless of query</t>
+        </is>
+      </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>integration</t>
+        </is>
+      </c>
+      <c r="D279" t="inlineStr">
+        <is>
+          <t>get_event_registry_entry</t>
+        </is>
+      </c>
+      <c r="E279" t="inlineStr">
+        <is>
+          <t>Fishy</t>
+        </is>
+      </c>
+      <c r="F279" t="inlineStr">
+        <is>
+          <t>Wrong filter field</t>
+        </is>
+      </c>
+      <c r="G279" t="inlineStr">
+        <is>
+          <t>Wave 1</t>
+        </is>
+      </c>
+      <c r="H279" t="inlineStr">
+        <is>
+          <t>Change encoded query from name=&lt;value&gt; to event_name=&lt;value&gt; on sysevent_register table.</t>
+        </is>
+      </c>
+      <c r="I279" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J279" t="inlineStr">
+        <is>
+          <t>Fork</t>
+        </is>
+      </c>
+      <c r="K279" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="L279" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="M279" t="inlineStr">
+        <is>
+          <t>sysevent_register uses event_name as the primary identifier, not name. Query with name= silently ignores filter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="n">
+        <v>18</v>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>register_event — event_name field empty on created record; sets 'name' instead of 'event_name'</t>
+        </is>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>integration</t>
+        </is>
+      </c>
+      <c r="D280" t="inlineStr">
+        <is>
+          <t>register_event</t>
+        </is>
+      </c>
+      <c r="E280" t="inlineStr">
+        <is>
+          <t>Fishy</t>
+        </is>
+      </c>
+      <c r="F280" t="inlineStr">
+        <is>
+          <t>Wrong field name</t>
+        </is>
+      </c>
+      <c r="G280" t="inlineStr">
+        <is>
+          <t>Wave 1</t>
+        </is>
+      </c>
+      <c r="H280" t="inlineStr">
+        <is>
+          <t>In createRecord payload, change key 'name' to 'event_name' to match the sysevent_register schema.</t>
+        </is>
+      </c>
+      <c r="I280" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J280" t="inlineStr">
+        <is>
+          <t>Fork</t>
+        </is>
+      </c>
+      <c r="K280" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="L280" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="M280" t="inlineStr">
+        <is>
+          <t>Record sys_id 0cafcb3b83e40310ad3cc4d0deaad3c9 created with empty event_name. Cleanup required on PDI.</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="n">
+        <v>19</v>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>list_homepages — Invalid table sys_ui_hp does not exist</t>
+        </is>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>performance</t>
+        </is>
+      </c>
+      <c r="D281" t="inlineStr">
+        <is>
+          <t>list_homepages</t>
+        </is>
+      </c>
+      <c r="E281" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="F281" t="inlineStr">
+        <is>
+          <t>Wrong table name</t>
+        </is>
+      </c>
+      <c r="G281" t="inlineStr">
+        <is>
+          <t>Wave 1</t>
+        </is>
+      </c>
+      <c r="H281" t="inlineStr">
+        <is>
+          <t>Correct table for homepages is sys_ui_homepage. Update the queryRecords call accordingly.</t>
+        </is>
+      </c>
+      <c r="I281" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J281" t="inlineStr">
+        <is>
+          <t>Fork</t>
+        </is>
+      </c>
+      <c r="K281" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="L281" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="M281" t="inlineStr">
+        <is>
+          <t>sys_ui_hp is not a ServiceNow table. Standard homepages are in sys_ui_homepage.</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="n">
+        <v>20</v>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>list_pa_jobs / get_pa_job — Invalid table pa_job does not exist</t>
+        </is>
+      </c>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>performance</t>
+        </is>
+      </c>
+      <c r="D282" t="inlineStr">
+        <is>
+          <t>list_pa_jobs, get_pa_job</t>
+        </is>
+      </c>
+      <c r="E282" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="F282" t="inlineStr">
+        <is>
+          <t>Wrong table name</t>
+        </is>
+      </c>
+      <c r="G282" t="inlineStr">
+        <is>
+          <t>Wave 1</t>
+        </is>
+      </c>
+      <c r="H282" t="inlineStr">
+        <is>
+          <t>The correct table for PA collection jobs is sysauto_pa_job. Update both handlers.</t>
+        </is>
+      </c>
+      <c r="I282" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J282" t="inlineStr">
+        <is>
+          <t>Fork</t>
+        </is>
+      </c>
+      <c r="K282" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="L282" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="M282" t="inlineStr">
+        <is>
+          <t>pa_job does not exist on standard ServiceNow instances. Confirmed INVALID_REQUEST on PDI.</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="n">
+        <v>21</v>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>export_properties — category filter silently ignored; returns all 500 properties</t>
+        </is>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>sys-properties</t>
+        </is>
+      </c>
+      <c r="D283" t="inlineStr">
+        <is>
+          <t>export_properties</t>
+        </is>
+      </c>
+      <c r="E283" t="inlineStr">
+        <is>
+          <t>Fishy</t>
+        </is>
+      </c>
+      <c r="F283" t="inlineStr">
+        <is>
+          <t>Wrong filter field</t>
+        </is>
+      </c>
+      <c r="G283" t="inlineStr">
+        <is>
+          <t>Wave 1</t>
+        </is>
+      </c>
+      <c r="H283" t="inlineStr">
+        <is>
+          <t>Verify the sys_properties field for category. It may be category (reference) requiring a sys_id rather than the category name string. Test with actual category sys_id or use sys_properties_category join.</t>
+        </is>
+      </c>
+      <c r="I283" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J283" t="inlineStr">
+        <is>
+          <t>Fork</t>
+        </is>
+      </c>
+      <c r="K283" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="L283" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="M283" t="inlineStr">
+        <is>
+          <t>PDI may have uncategorised properties only, making this hard to isolate. Verify on production-like instance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="n">
+        <v>22</v>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>get_va_conversation — Invalid table sys_cs_conversation_message does not exist</t>
+        </is>
+      </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>va</t>
+        </is>
+      </c>
+      <c r="D284" t="inlineStr">
+        <is>
+          <t>get_va_conversation</t>
+        </is>
+      </c>
+      <c r="E284" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="F284" t="inlineStr">
+        <is>
+          <t>Wrong table name</t>
+        </is>
+      </c>
+      <c r="G284" t="inlineStr">
+        <is>
+          <t>Wave 1</t>
+        </is>
+      </c>
+      <c r="H284" t="inlineStr">
+        <is>
+          <t>VA conversation messages are in sys_cs_chat_queue_message or similar. Investigate correct table via sys_db_object query on a licensed instance.</t>
+        </is>
+      </c>
+      <c r="I284" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J284" t="inlineStr">
+        <is>
+          <t>Fork</t>
+        </is>
+      </c>
+      <c r="K284" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="L284" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="M284" t="inlineStr">
+        <is>
+          <t>sys_cs_conversation_message is not a standard table. Correct table may require Conversational Platform license.</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="n">
+        <v>23</v>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>list_va_categories — Invalid table sys_cs_category does not exist</t>
+        </is>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>va</t>
+        </is>
+      </c>
+      <c r="D285" t="inlineStr">
+        <is>
+          <t>list_va_categories</t>
+        </is>
+      </c>
+      <c r="E285" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="F285" t="inlineStr">
+        <is>
+          <t>Wrong table name</t>
+        </is>
+      </c>
+      <c r="G285" t="inlineStr">
+        <is>
+          <t>Wave 1</t>
+        </is>
+      </c>
+      <c r="H285" t="inlineStr">
+        <is>
+          <t>VA categories use sys_cs_category_config or are embedded in topic records. Verify correct table on a licensed NLU instance.</t>
+        </is>
+      </c>
+      <c r="I285" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J285" t="inlineStr">
+        <is>
+          <t>Fork</t>
+        </is>
+      </c>
+      <c r="K285" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="L285" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="M285" t="inlineStr">
+        <is>
+          <t>sys_cs_category is not a standard ServiceNow table. Category data may be stored differently in newer VA versions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="n">
+        <v>24</v>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>get_performance_analytics — fallback hits invalid table pa_job_log</t>
+        </is>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>reporting</t>
+        </is>
+      </c>
+      <c r="D286" t="inlineStr">
+        <is>
+          <t>get_performance_analytics</t>
+        </is>
+      </c>
+      <c r="E286" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="F286" t="inlineStr">
+        <is>
+          <t>Wrong table name</t>
+        </is>
+      </c>
+      <c r="G286" t="inlineStr">
+        <is>
+          <t>Wave 1</t>
+        </is>
+      </c>
+      <c r="H286" t="inlineStr">
+        <is>
+          <t>Remove the pa_job_log fallback entirely. If the PA widget API call fails, return an error rather than querying a non-existent table.</t>
+        </is>
+      </c>
+      <c r="I286" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J286" t="inlineStr">
+        <is>
+          <t>Fork</t>
+        </is>
+      </c>
+      <c r="K286" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="L286" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="M286" t="inlineStr">
+        <is>
+          <t>Tool tries /api/now/pa/widget/ first; on error falls back to pa_job_log which does not exist. pa_job_log is not a standard table.</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="n">
+        <v>25</v>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>ml_model_training_history — Invalid table ml_solution_version does not exist</t>
+        </is>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>ml</t>
+        </is>
+      </c>
+      <c r="D287" t="inlineStr">
+        <is>
+          <t>ml_model_training_history</t>
+        </is>
+      </c>
+      <c r="E287" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="F287" t="inlineStr">
+        <is>
+          <t>Wrong table name</t>
+        </is>
+      </c>
+      <c r="G287" t="inlineStr">
+        <is>
+          <t>Wave 1</t>
+        </is>
+      </c>
+      <c r="H287" t="inlineStr">
+        <is>
+          <t>Correct table for PI model versions/training history is ml_solution (query training-related fields) or ml_train_result. Verify on a PI-licensed instance.</t>
+        </is>
+      </c>
+      <c r="I287" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J287" t="inlineStr">
+        <is>
+          <t>Fork</t>
+        </is>
+      </c>
+      <c r="K287" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="L287" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="M287" t="inlineStr">
+        <is>
+          <t>ml_solution_version is not a standard ServiceNow table. Training history may be in ml_solution or a plugin-specific table.</t>
         </is>
       </c>
     </row>

</xml_diff>